<commit_message>
Se le hace mantenimiento al proyecto.
</commit_message>
<xml_diff>
--- a/src/test/resources/excel/DatosPruebaWeb.xlsx
+++ b/src/test/resources/excel/DatosPruebaWeb.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automatizacion\Practivas Automatización Web\PruebaTenicaAutomatizacionWeb\src\test\resources\excel\"/>
     </mc:Choice>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="81">
   <si>
     <t>Numero de cedula</t>
   </si>
@@ -263,12 +263,16 @@
   </si>
   <si>
     <t>Billetera en cuero rojo achiote</t>
+  </si>
+  <si>
+    <t>PQRS-01a13c78-1e72-7716</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="0"/>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -734,7 +738,7 @@
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="4" max="4" width="37.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="37.7265625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
@@ -938,7 +942,7 @@
       <c r="J1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" t="s" s="0">
         <v>76</v>
       </c>
     </row>
@@ -973,8 +977,8 @@
       <c r="J2" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="K2" t="s">
-        <v>77</v>
+      <c r="K2" t="s" s="0">
+        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>